<commit_message>
feat: update excel format and 7d average for BTC
</commit_message>
<xml_diff>
--- a/crypto_volume.xlsx
+++ b/crypto_volume.xlsx
@@ -413,299 +413,236 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Bitkub</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ave. daily vol. (THB)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Binance TH</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ave. daily vol. (THB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>THB_USDT</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>354658771.72</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>USDTTHB</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>298158638.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>THB_BTC</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>69595143.01000001</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BTCTHB</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>54634259.87466</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>THB_ETH</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>14733990.67</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VELOTHB</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1566785.1844</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>THB_KUB</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>8652846.640000001</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>XRPTHB</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>530097.1267</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>THB_XRP</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>8554651.029999999</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ETHTHB</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>365463.454</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Exchange</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Rank</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Symbol</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Volume (THB)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Price (THB)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Binance TH</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>THB_USDT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>THB_BTC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>THB_BTC 7d-Avg</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>THB_ETH</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>THB_KUB</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>THB_XRP</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>USDTTHB</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>502390836.85</v>
-      </c>
-      <c r="F2" t="n">
-        <v>33.11</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Binance TH</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>BTCTHB</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>63050072.75102</v>
-      </c>
-      <c r="F3" t="n">
-        <v>2078248</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Binance TH</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>BTCTHB 7d-Avg</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>VELOTHB</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>1963361.639</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.1086</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Binance TH</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>XRPTHB</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>734427.0186</v>
-      </c>
-      <c r="F5" t="n">
-        <v>33.22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Binance TH</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SOLTHB</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>375017.7144</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2506.85</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Bitkub</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>THB_USDT</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>393600320.76</v>
-      </c>
-      <c r="F7" t="n">
-        <v>33.11</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Bitkub</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>THB_BTC</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>139379317.8</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2078284.52</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Bitkub</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>THB_ETH</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>27173995.54</v>
-      </c>
-      <c r="F9" t="n">
-        <v>62000.05</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Bitkub</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>4</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>THB_XRP</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>12035607.92</v>
-      </c>
-      <c r="F10" t="n">
-        <v>33.18</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-14 16:39:06</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Bitkub</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>THB_USDC</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>7456966.86</v>
-      </c>
-      <c r="F11" t="n">
-        <v>33.11</v>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>ETHTHB</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B14" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2082634.88</v>
+      </c>
+      <c r="E14" t="n">
+        <v>62175.42</v>
+      </c>
+      <c r="F14" t="n">
+        <v>15.71</v>
+      </c>
+      <c r="G14" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="H14" t="n">
+        <v>33.05</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2082026</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.1015</v>
+      </c>
+      <c r="L14" t="n">
+        <v>33.09</v>
+      </c>
+      <c r="M14" t="n">
+        <v>62201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: track history for all coins and add 7d avg for BTC
</commit_message>
<xml_diff>
--- a/crypto_volume.xlsx
+++ b/crypto_volume.xlsx
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,16 +448,16 @@
           <t>THB_USDT</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>354658771.72</v>
+      <c r="C2" s="1" t="n">
+        <v>353708238.6</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>USDTTHB</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>298158638.7</v>
+      <c r="E2" s="1" t="n">
+        <v>295567718.67</v>
       </c>
     </row>
     <row r="3">
@@ -468,16 +469,16 @@
           <t>THB_BTC</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>69595143.01000001</v>
+      <c r="C3" s="1" t="n">
+        <v>69559195.08</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>BTCTHB</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>54634259.87466</v>
+      <c r="E3" s="1" t="n">
+        <v>54186128.94003</v>
       </c>
     </row>
     <row r="4">
@@ -489,16 +490,16 @@
           <t>THB_ETH</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>14733990.67</v>
+      <c r="C4" s="1" t="n">
+        <v>14751066.16</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>VELOTHB</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>1566785.1844</v>
+      <c r="E4" s="1" t="n">
+        <v>1564635.1658</v>
       </c>
     </row>
     <row r="5">
@@ -510,16 +511,16 @@
           <t>THB_KUB</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>8652846.640000001</v>
+      <c r="C5" s="1" t="n">
+        <v>8683443.720000001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>XRPTHB</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>530097.1267</v>
+      <c r="E5" s="1" t="n">
+        <v>685073.3212</v>
       </c>
     </row>
     <row r="6">
@@ -531,15 +532,15 @@
           <t>THB_XRP</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>8554651.029999999</v>
+      <c r="C6" s="1" t="n">
+        <v>8611087.689999999</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>ETHTHB</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="1" t="n">
         <v>365463.454</v>
       </c>
     </row>
@@ -614,34 +615,34 @@
       <c r="A14" t="n">
         <v>16</v>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="1" t="n">
+        <v>33.07</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>2082299.99</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>62181.42</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="G14" s="1" t="n">
         <v>33.06</v>
       </c>
-      <c r="C14" t="n">
-        <v>2082634.88</v>
-      </c>
-      <c r="E14" t="n">
-        <v>62175.42</v>
-      </c>
-      <c r="F14" t="n">
-        <v>15.71</v>
-      </c>
-      <c r="G14" t="n">
+      <c r="H14" s="1" t="n">
         <v>33.06</v>
       </c>
-      <c r="H14" t="n">
-        <v>33.05</v>
-      </c>
-      <c r="I14" t="n">
-        <v>2082026</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0.1015</v>
-      </c>
-      <c r="L14" t="n">
-        <v>33.09</v>
-      </c>
-      <c r="M14" t="n">
+      <c r="I14" s="1" t="n">
+        <v>2082425</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>0.1018</v>
+      </c>
+      <c r="L14" s="1" t="n">
+        <v>33.08</v>
+      </c>
+      <c r="M14" s="1" t="n">
         <v>62201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: change historical data from price to volume
</commit_message>
<xml_diff>
--- a/crypto_volume.xlsx
+++ b/crypto_volume.xlsx
@@ -449,7 +449,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>353708238.6</v>
+        <v>555935973.22</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>295567718.67</v>
+        <v>349253017.36</v>
       </c>
     </row>
     <row r="3">
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>69559195.08</v>
+        <v>83947187.86</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="E3" s="1" t="n">
-        <v>54186128.94003</v>
+        <v>55147671.45308</v>
       </c>
     </row>
     <row r="4">
@@ -491,15 +491,15 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>14751066.16</v>
+        <v>33938402.4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>VELOTHB</t>
+          <t>ETHTHB</t>
         </is>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1564635.1658</v>
+        <v>1214584.6106</v>
       </c>
     </row>
     <row r="5">
@@ -508,19 +508,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>THB_KUB</t>
+          <t>THB_XRP</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>8683443.720000001</v>
+        <v>15978823.17</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>XRPTHB</t>
+          <t>VELOTHB</t>
         </is>
       </c>
       <c r="E5" s="1" t="n">
-        <v>685073.3212</v>
+        <v>1133712.6956</v>
       </c>
     </row>
     <row r="6">
@@ -529,19 +529,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>THB_XRP</t>
+          <t>THB_KUB</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>8611087.689999999</v>
+        <v>8714676.98</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ETHTHB</t>
+          <t>XRPTHB</t>
         </is>
       </c>
       <c r="E6" s="1" t="n">
-        <v>365463.454</v>
+        <v>1100220.0746</v>
       </c>
     </row>
     <row r="13">
@@ -572,14 +572,14 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>THB_XRP</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>THB_KUB</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>THB_XRP</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>USDTTHB</t>
@@ -597,53 +597,53 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
+          <t>ETHTHB</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>VELOTHB</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>XRPTHB</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>ETHTHB</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>33.07</v>
+        <v>555935973.22</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>2082299.99</v>
+        <v>83947187.86</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>62181.42</v>
+        <v>33938402.4</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>15.61</v>
+        <v>15978823.17</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>33.06</v>
+        <v>8714676.98</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>33.06</v>
+        <v>349253017.36</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>2082425</v>
+        <v>55147671.45308</v>
       </c>
       <c r="K14" s="1" t="n">
-        <v>0.1018</v>
+        <v>1214584.6106</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>33.08</v>
+        <v>1133712.6956</v>
       </c>
       <c r="M14" s="1" t="n">
-        <v>62201</v>
+        <v>1100220.0746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add column gap between Bitkub and Binance TH groups
</commit_message>
<xml_diff>
--- a/crypto_volume.xlsx
+++ b/crypto_volume.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:GQ15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,6 +438,26 @@
           <t>Ave. daily vol. (THB)</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Bitkub</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Ave. daily vol. (THB)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Binance TH</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Ave. daily vol. (THB)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -449,7 +469,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>555935973.22</v>
+        <v>558774049.83</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -457,7 +477,23 @@
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>349253017.36</v>
+        <v>349792699.51</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>THB_USDT</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>558763983.42</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>USDTTHB</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="n">
+        <v>349792699.51</v>
       </c>
     </row>
     <row r="3">
@@ -470,7 +506,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>83947187.86</v>
+        <v>84235751.65000001</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -478,7 +514,23 @@
         </is>
       </c>
       <c r="E3" s="1" t="n">
-        <v>55147671.45308</v>
+        <v>55889180.66205</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>THB_BTC</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>84235751.65000001</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>BTCTHB</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>55889180.66205</v>
       </c>
     </row>
     <row r="4">
@@ -491,7 +543,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>33938402.4</v>
+        <v>33819519.53</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -499,7 +551,23 @@
         </is>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1214584.6106</v>
+        <v>1234378.8297</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>THB_ETH</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>33822631.66</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ETHTHB</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>1234378.8297</v>
       </c>
     </row>
     <row r="5">
@@ -512,7 +580,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>15978823.17</v>
+        <v>16206221.05</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -520,7 +588,23 @@
         </is>
       </c>
       <c r="E5" s="1" t="n">
-        <v>1133712.6956</v>
+        <v>1125889.5078</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>THB_XRP</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>16206221.05</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>VELOTHB</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>1125889.5078</v>
       </c>
     </row>
     <row r="6">
@@ -533,7 +617,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>8714676.98</v>
+        <v>8641198.48</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -541,7 +625,23 @@
         </is>
       </c>
       <c r="E6" s="1" t="n">
-        <v>1100220.0746</v>
+        <v>1093867.338</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>THB_KUB</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>8641198.48</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>XRPTHB</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>1093867.338</v>
       </c>
     </row>
     <row r="13">
@@ -580,32 +680,32 @@
           <t>THB_KUB</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>USDTTHB</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>BTCTHB</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>BTCTHB 7d-Avg</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>ETHTHB</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>VELOTHB</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>XRPTHB</t>
         </is>
@@ -616,34 +716,69 @@
         <v>17</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>555935973.22</v>
+        <v>558763983.42</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>83947187.86</v>
+        <v>84235751.65000001</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>33938402.4</v>
+        <v>33822631.66</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>15978823.17</v>
+        <v>16206221.05</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>8714676.98</v>
-      </c>
-      <c r="H14" s="1" t="n">
-        <v>349253017.36</v>
+        <v>8641198.48</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>55147671.45308</v>
-      </c>
-      <c r="K14" s="1" t="n">
-        <v>1214584.6106</v>
+        <v>349792699.51</v>
+      </c>
+      <c r="J14" s="1" t="n">
+        <v>55889180.66205</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>1133712.6956</v>
+        <v>1234378.8297</v>
       </c>
       <c r="M14" s="1" t="n">
-        <v>1100220.0746</v>
+        <v>1125889.5078</v>
+      </c>
+      <c r="N14" s="1" t="n">
+        <v>1093867.338</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>17</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>558774049.83</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>84235751.65000001</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>33819519.53</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>16206221.05</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>8641198.48</v>
+      </c>
+      <c r="I15" s="1" t="n">
+        <v>349792699.51</v>
+      </c>
+      <c r="J15" s="1" t="n">
+        <v>55889180.66205</v>
+      </c>
+      <c r="L15" s="1" t="n">
+        <v>1234378.8297</v>
+      </c>
+      <c r="M15" s="1" t="n">
+        <v>1125889.5078</v>
+      </c>
+      <c r="N15" s="1" t="n">
+        <v>1093867.338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: change cron schedule to avoid top-of-the-hour delays
</commit_message>
<xml_diff>
--- a/crypto_volume.xlsx
+++ b/crypto_volume.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>574690297.36</v>
+        <v>568660713.29</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>467330717.69</v>
+        <v>477159198.56</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -489,7 +489,15 @@
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>11418675.23511377</v>
+        <v>11362893.17644277</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>BTCTHB</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>22777811.28</v>
       </c>
     </row>
     <row r="3">
@@ -502,7 +510,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>226027491.92</v>
+        <v>230172684.85</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -510,7 +518,7 @@
         </is>
       </c>
       <c r="F3" s="1" t="n">
-        <v>56626600.72849</v>
+        <v>59431221.008</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -518,7 +526,15 @@
         </is>
       </c>
       <c r="I3" s="1" t="n">
-        <v>5915900.034764385</v>
+        <v>5798165.383009525</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>XRPTHB</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>3656214.5</v>
       </c>
     </row>
     <row r="4">
@@ -531,7 +547,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>110109964.92</v>
+        <v>111501034.51</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -539,7 +555,7 @@
         </is>
       </c>
       <c r="F4" s="1" t="n">
-        <v>13094292.6231</v>
+        <v>12347424.0953</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -547,7 +563,15 @@
         </is>
       </c>
       <c r="I4" s="1" t="n">
-        <v>3556224.796734105</v>
+        <v>3595761.256052385</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ETHTHB</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>1295063.04</v>
       </c>
     </row>
     <row r="5">
@@ -560,7 +584,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>74029329.95</v>
+        <v>72974131.79000001</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -568,7 +592,7 @@
         </is>
       </c>
       <c r="F5" s="1" t="n">
-        <v>8661351.4428</v>
+        <v>8972833.5349</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -577,6 +601,14 @@
       </c>
       <c r="I5" s="1" t="n">
         <v>759551.87093175</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>SOLTHB</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>1113927.77</v>
       </c>
     </row>
     <row r="6">
@@ -589,7 +621,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>37196128.88</v>
+        <v>38907350.08</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -597,7 +629,7 @@
         </is>
       </c>
       <c r="F6" s="1" t="n">
-        <v>3115484.7788</v>
+        <v>3269370.7132</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -605,7 +637,15 @@
         </is>
       </c>
       <c r="I6" s="1" t="n">
-        <v>714843.6512889932</v>
+        <v>576305.3392889932</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>BCHTHB</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>465985.55</v>
       </c>
     </row>
     <row r="7"/>
@@ -622,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW2"/>
+  <dimension ref="A1:BXW3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4175,6 +4215,1337 @@
         <v>0</v>
       </c>
       <c r="QB2" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>568660713.29</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>230172684.85</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>111501034.51</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>72974131.79000001</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>38907350.08</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>33144379.36</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>11977123.27</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>11580035.25</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>10071884.83</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>8682439.02</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <v>10799962.4</v>
+      </c>
+      <c r="N3" s="1" t="n">
+        <v>8177609.11</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>7156639.01</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>7406149.72</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>6596483.82</v>
+      </c>
+      <c r="R3" s="1" t="n">
+        <v>6145877.72</v>
+      </c>
+      <c r="S3" s="1" t="n">
+        <v>6131176.94</v>
+      </c>
+      <c r="T3" s="1" t="n">
+        <v>5775203.51</v>
+      </c>
+      <c r="U3" s="1" t="n">
+        <v>5190318.49</v>
+      </c>
+      <c r="V3" s="1" t="n">
+        <v>4065809.69</v>
+      </c>
+      <c r="W3" s="1" t="n">
+        <v>3332110.98</v>
+      </c>
+      <c r="X3" s="1" t="n">
+        <v>4077416.43</v>
+      </c>
+      <c r="Y3" s="1" t="n">
+        <v>4029103.77</v>
+      </c>
+      <c r="Z3" s="1" t="n">
+        <v>3560406.86</v>
+      </c>
+      <c r="AA3" s="1" t="n">
+        <v>3341772.76</v>
+      </c>
+      <c r="AB3" s="1" t="n">
+        <v>3404112.36</v>
+      </c>
+      <c r="AC3" s="1" t="n">
+        <v>3692783.24</v>
+      </c>
+      <c r="AD3" s="1" t="n">
+        <v>3163337.51</v>
+      </c>
+      <c r="AE3" s="1" t="n">
+        <v>2950372.97</v>
+      </c>
+      <c r="AF3" s="1" t="n">
+        <v>2763123.05</v>
+      </c>
+      <c r="AG3" s="1" t="n">
+        <v>2204654.73</v>
+      </c>
+      <c r="AH3" s="1" t="n">
+        <v>2369395.92</v>
+      </c>
+      <c r="AI3" s="1" t="n">
+        <v>2125534.84</v>
+      </c>
+      <c r="AJ3" s="1" t="n">
+        <v>1939655.56</v>
+      </c>
+      <c r="AK3" s="1" t="n">
+        <v>1686357.36</v>
+      </c>
+      <c r="AL3" s="1" t="n">
+        <v>1973409.27</v>
+      </c>
+      <c r="AM3" s="1" t="n">
+        <v>1587235.59</v>
+      </c>
+      <c r="AN3" s="1" t="n">
+        <v>894982.11</v>
+      </c>
+      <c r="AO3" s="1" t="n">
+        <v>1517274.92</v>
+      </c>
+      <c r="AP3" s="1" t="n">
+        <v>1711067.44</v>
+      </c>
+      <c r="AQ3" s="1" t="n">
+        <v>1503267.29</v>
+      </c>
+      <c r="AR3" s="1" t="n">
+        <v>1512573.4</v>
+      </c>
+      <c r="AS3" s="1" t="n">
+        <v>1434386.8</v>
+      </c>
+      <c r="AT3" s="1" t="n">
+        <v>1301323.68</v>
+      </c>
+      <c r="AU3" s="1" t="n">
+        <v>1369240.07</v>
+      </c>
+      <c r="AV3" s="1" t="n">
+        <v>1375458.9</v>
+      </c>
+      <c r="AW3" s="1" t="n">
+        <v>1513007</v>
+      </c>
+      <c r="AX3" s="1" t="n">
+        <v>1351206.18</v>
+      </c>
+      <c r="AY3" s="1" t="n">
+        <v>1090368.94</v>
+      </c>
+      <c r="AZ3" s="1" t="n">
+        <v>1096439.97</v>
+      </c>
+      <c r="BA3" s="1" t="n">
+        <v>1064297.97</v>
+      </c>
+      <c r="BB3" s="1" t="n">
+        <v>1143562.45</v>
+      </c>
+      <c r="BC3" s="1" t="n">
+        <v>1238748.59</v>
+      </c>
+      <c r="BD3" s="1" t="n">
+        <v>1033588.43</v>
+      </c>
+      <c r="BE3" s="1" t="n">
+        <v>928864.66</v>
+      </c>
+      <c r="BF3" s="1" t="n">
+        <v>879680.92</v>
+      </c>
+      <c r="BG3" s="1" t="n">
+        <v>867824.39</v>
+      </c>
+      <c r="BH3" s="1" t="n">
+        <v>862014.58</v>
+      </c>
+      <c r="BI3" s="1" t="n">
+        <v>863504.4300000001</v>
+      </c>
+      <c r="BJ3" s="1" t="n">
+        <v>806717.8</v>
+      </c>
+      <c r="BK3" s="1" t="n">
+        <v>893236.64</v>
+      </c>
+      <c r="BL3" s="1" t="n">
+        <v>998049.47</v>
+      </c>
+      <c r="BM3" s="1" t="n">
+        <v>804382.71</v>
+      </c>
+      <c r="BN3" s="1" t="n">
+        <v>716464.6899999999</v>
+      </c>
+      <c r="BO3" s="1" t="n">
+        <v>718904.38</v>
+      </c>
+      <c r="BP3" s="1" t="n">
+        <v>639033.9399999999</v>
+      </c>
+      <c r="BQ3" s="1" t="n">
+        <v>640818.52</v>
+      </c>
+      <c r="BR3" s="1" t="n">
+        <v>606043.35</v>
+      </c>
+      <c r="BS3" s="1" t="n">
+        <v>545075.72</v>
+      </c>
+      <c r="BT3" s="1" t="n">
+        <v>693630.13</v>
+      </c>
+      <c r="BU3" s="1" t="n">
+        <v>564758.71</v>
+      </c>
+      <c r="BV3" s="1" t="n">
+        <v>608929.02</v>
+      </c>
+      <c r="BW3" s="1" t="n">
+        <v>538879.3100000001</v>
+      </c>
+      <c r="BX3" s="1" t="n">
+        <v>573376.49</v>
+      </c>
+      <c r="BY3" s="1" t="n">
+        <v>513730.95</v>
+      </c>
+      <c r="BZ3" s="1" t="n">
+        <v>432453.18</v>
+      </c>
+      <c r="CA3" s="1" t="n">
+        <v>427907.93</v>
+      </c>
+      <c r="CB3" s="1" t="n">
+        <v>421370.68</v>
+      </c>
+      <c r="CC3" s="1" t="n">
+        <v>483106.95</v>
+      </c>
+      <c r="CD3" s="1" t="n">
+        <v>407036.04</v>
+      </c>
+      <c r="CE3" s="1" t="n">
+        <v>378119.94</v>
+      </c>
+      <c r="CF3" s="1" t="n">
+        <v>371827.31</v>
+      </c>
+      <c r="CG3" s="1" t="n">
+        <v>1113419.11</v>
+      </c>
+      <c r="CH3" s="1" t="n">
+        <v>362350.43</v>
+      </c>
+      <c r="CI3" s="1" t="n">
+        <v>363948.84</v>
+      </c>
+      <c r="CJ3" s="1" t="n">
+        <v>363905.89</v>
+      </c>
+      <c r="CK3" s="1" t="n">
+        <v>340285.71</v>
+      </c>
+      <c r="CL3" s="1" t="n">
+        <v>332264.97</v>
+      </c>
+      <c r="CM3" s="1" t="n">
+        <v>305083.15</v>
+      </c>
+      <c r="CN3" s="1" t="n">
+        <v>273464.17</v>
+      </c>
+      <c r="CO3" s="1" t="n">
+        <v>781362.66</v>
+      </c>
+      <c r="CP3" s="1" t="n">
+        <v>194527.17</v>
+      </c>
+      <c r="CQ3" s="1" t="n">
+        <v>286267.5</v>
+      </c>
+      <c r="CR3" s="1" t="n">
+        <v>237564.35</v>
+      </c>
+      <c r="CS3" s="1" t="n">
+        <v>266224.24</v>
+      </c>
+      <c r="CT3" s="1" t="n">
+        <v>261778.9</v>
+      </c>
+      <c r="CU3" s="1" t="n">
+        <v>246667.8</v>
+      </c>
+      <c r="CV3" s="1" t="n">
+        <v>296079.68</v>
+      </c>
+      <c r="CW3" s="1" t="n">
+        <v>243211.78</v>
+      </c>
+      <c r="CX3" s="1" t="n">
+        <v>238788.96</v>
+      </c>
+      <c r="CY3" s="1" t="n">
+        <v>236054.04</v>
+      </c>
+      <c r="CZ3" s="1" t="n">
+        <v>232357.6</v>
+      </c>
+      <c r="DA3" s="1" t="n">
+        <v>223955.74</v>
+      </c>
+      <c r="DB3" s="1" t="n">
+        <v>215864.86</v>
+      </c>
+      <c r="DC3" s="1" t="n">
+        <v>210972.48</v>
+      </c>
+      <c r="DD3" s="1" t="n">
+        <v>210647.2</v>
+      </c>
+      <c r="DE3" s="1" t="n">
+        <v>204713.72</v>
+      </c>
+      <c r="DF3" s="1" t="n">
+        <v>196756.47</v>
+      </c>
+      <c r="DG3" s="1" t="n">
+        <v>125216.39</v>
+      </c>
+      <c r="DH3" s="1" t="n">
+        <v>187286.64</v>
+      </c>
+      <c r="DI3" s="1" t="n">
+        <v>183098.03</v>
+      </c>
+      <c r="DJ3" s="1" t="n">
+        <v>207774.83</v>
+      </c>
+      <c r="DK3" s="1" t="n">
+        <v>165952.53</v>
+      </c>
+      <c r="DL3" s="1" t="n">
+        <v>163871.54</v>
+      </c>
+      <c r="DM3" s="1" t="n">
+        <v>166433.16</v>
+      </c>
+      <c r="DN3" s="1" t="n">
+        <v>215715.14</v>
+      </c>
+      <c r="DO3" s="1" t="n">
+        <v>146580.59</v>
+      </c>
+      <c r="DP3" s="1" t="n">
+        <v>153334.24</v>
+      </c>
+      <c r="DQ3" s="1" t="n">
+        <v>150055.85</v>
+      </c>
+      <c r="DR3" s="1" t="n">
+        <v>148333.96</v>
+      </c>
+      <c r="DS3" s="1" t="n">
+        <v>144183.72</v>
+      </c>
+      <c r="DT3" s="1" t="n">
+        <v>290587.99</v>
+      </c>
+      <c r="DU3" s="1" t="n">
+        <v>135243.2</v>
+      </c>
+      <c r="DV3" s="1" t="n">
+        <v>128842.15</v>
+      </c>
+      <c r="DW3" s="1" t="n">
+        <v>156516.8</v>
+      </c>
+      <c r="DX3" s="1" t="n">
+        <v>137876.66</v>
+      </c>
+      <c r="DY3" s="1" t="n">
+        <v>125985.42</v>
+      </c>
+      <c r="DZ3" s="1" t="n">
+        <v>118854.8</v>
+      </c>
+      <c r="EA3" s="1" t="n">
+        <v>138669.02</v>
+      </c>
+      <c r="EB3" s="1" t="n">
+        <v>115816.67</v>
+      </c>
+      <c r="EC3" s="1" t="n">
+        <v>107811.02</v>
+      </c>
+      <c r="ED3" s="1" t="n">
+        <v>107950.9</v>
+      </c>
+      <c r="EE3" s="1" t="n">
+        <v>106573.26</v>
+      </c>
+      <c r="EF3" s="1" t="n">
+        <v>104382.5</v>
+      </c>
+      <c r="EG3" s="1" t="n">
+        <v>102315.68</v>
+      </c>
+      <c r="EH3" s="1" t="n">
+        <v>103215.28</v>
+      </c>
+      <c r="EI3" s="1" t="n">
+        <v>21036.29</v>
+      </c>
+      <c r="EJ3" s="1" t="n">
+        <v>82848.03</v>
+      </c>
+      <c r="EK3" s="1" t="n">
+        <v>145671.33</v>
+      </c>
+      <c r="EL3" s="1" t="n">
+        <v>97497.53</v>
+      </c>
+      <c r="EM3" s="1" t="n">
+        <v>102231.33</v>
+      </c>
+      <c r="EN3" s="1" t="n">
+        <v>92954.91</v>
+      </c>
+      <c r="EO3" s="1" t="n">
+        <v>87769.41</v>
+      </c>
+      <c r="EP3" s="1" t="n">
+        <v>126988.33</v>
+      </c>
+      <c r="EQ3" s="1" t="n">
+        <v>83717.39999999999</v>
+      </c>
+      <c r="ER3" s="1" t="n">
+        <v>91828.47</v>
+      </c>
+      <c r="ES3" s="1" t="n">
+        <v>96509.25999999999</v>
+      </c>
+      <c r="ET3" s="1" t="n">
+        <v>77953.46000000001</v>
+      </c>
+      <c r="EU3" s="1" t="n">
+        <v>75420.2</v>
+      </c>
+      <c r="EV3" s="1" t="n">
+        <v>55275.78</v>
+      </c>
+      <c r="EW3" s="1" t="n">
+        <v>32885.7</v>
+      </c>
+      <c r="EX3" s="1" t="n">
+        <v>76072.67</v>
+      </c>
+      <c r="EY3" s="1" t="n">
+        <v>69787.16</v>
+      </c>
+      <c r="EZ3" s="1" t="n">
+        <v>67759.47</v>
+      </c>
+      <c r="FA3" s="1" t="n">
+        <v>66407.73</v>
+      </c>
+      <c r="FB3" s="1" t="n">
+        <v>66124.87</v>
+      </c>
+      <c r="FC3" s="1" t="n">
+        <v>65676.05</v>
+      </c>
+      <c r="FD3" s="1" t="n">
+        <v>65539.53</v>
+      </c>
+      <c r="FE3" s="1" t="n">
+        <v>65190.88</v>
+      </c>
+      <c r="FF3" s="1" t="n">
+        <v>65548.62</v>
+      </c>
+      <c r="FG3" s="1" t="n">
+        <v>67113.61</v>
+      </c>
+      <c r="FH3" s="1" t="n">
+        <v>63512.76</v>
+      </c>
+      <c r="FI3" s="1" t="n">
+        <v>62357.75</v>
+      </c>
+      <c r="FJ3" s="1" t="n">
+        <v>61598.86</v>
+      </c>
+      <c r="FK3" s="1" t="n">
+        <v>41580.04</v>
+      </c>
+      <c r="FL3" s="1" t="n">
+        <v>58877.91</v>
+      </c>
+      <c r="FM3" s="1" t="n">
+        <v>60758.91</v>
+      </c>
+      <c r="FN3" s="1" t="n">
+        <v>60093.12</v>
+      </c>
+      <c r="FO3" s="1" t="n">
+        <v>496.99</v>
+      </c>
+      <c r="FP3" s="1" t="n">
+        <v>59065</v>
+      </c>
+      <c r="FQ3" s="1" t="n">
+        <v>81321.53999999999</v>
+      </c>
+      <c r="FR3" s="1" t="n">
+        <v>56209.17</v>
+      </c>
+      <c r="FS3" s="1" t="n">
+        <v>68464.27</v>
+      </c>
+      <c r="FT3" s="1" t="n">
+        <v>55803.1</v>
+      </c>
+      <c r="FU3" s="1" t="n">
+        <v>54822.34</v>
+      </c>
+      <c r="FV3" s="1" t="n">
+        <v>33556.27</v>
+      </c>
+      <c r="FW3" s="1" t="n">
+        <v>50625.14</v>
+      </c>
+      <c r="FX3" s="1" t="n">
+        <v>61289.23</v>
+      </c>
+      <c r="FY3" s="1" t="n">
+        <v>52681.62</v>
+      </c>
+      <c r="FZ3" s="1" t="n">
+        <v>51529.01</v>
+      </c>
+      <c r="GA3" s="1" t="n">
+        <v>49106.02</v>
+      </c>
+      <c r="GB3" s="1" t="n">
+        <v>48557.65</v>
+      </c>
+      <c r="GC3" s="1" t="n">
+        <v>48549.24</v>
+      </c>
+      <c r="GD3" s="1" t="n">
+        <v>47945.12</v>
+      </c>
+      <c r="GE3" s="1" t="n">
+        <v>48806.15</v>
+      </c>
+      <c r="GF3" s="1" t="n">
+        <v>47658.44</v>
+      </c>
+      <c r="GG3" s="1" t="n">
+        <v>46083.73</v>
+      </c>
+      <c r="GH3" s="1" t="n">
+        <v>45235.28</v>
+      </c>
+      <c r="GI3" s="1" t="n">
+        <v>45057.51</v>
+      </c>
+      <c r="GJ3" s="1" t="n">
+        <v>43539.13</v>
+      </c>
+      <c r="GK3" s="1" t="n">
+        <v>42842.24</v>
+      </c>
+      <c r="GL3" s="1" t="n">
+        <v>42266.15</v>
+      </c>
+      <c r="GM3" s="1" t="n">
+        <v>41818.55</v>
+      </c>
+      <c r="GN3" s="1" t="n">
+        <v>40923.3</v>
+      </c>
+      <c r="GO3" s="1" t="n">
+        <v>40616.23</v>
+      </c>
+      <c r="GP3" s="1" t="n">
+        <v>38922.98</v>
+      </c>
+      <c r="GQ3" s="1" t="n">
+        <v>38992.08</v>
+      </c>
+      <c r="GR3" s="1" t="n">
+        <v>38766.35</v>
+      </c>
+      <c r="GS3" s="1" t="n">
+        <v>37911.35</v>
+      </c>
+      <c r="GT3" s="1" t="n">
+        <v>38443.95</v>
+      </c>
+      <c r="GU3" s="1" t="n">
+        <v>37680.31</v>
+      </c>
+      <c r="GV3" s="1" t="n">
+        <v>37119.24</v>
+      </c>
+      <c r="GW3" s="1" t="n">
+        <v>36869.97</v>
+      </c>
+      <c r="GX3" s="1" t="n">
+        <v>36764.69</v>
+      </c>
+      <c r="GY3" s="1" t="n">
+        <v>35073.23</v>
+      </c>
+      <c r="GZ3" s="1" t="n">
+        <v>27346.51</v>
+      </c>
+      <c r="HA3" s="1" t="n">
+        <v>31393.39</v>
+      </c>
+      <c r="HB3" s="1" t="n">
+        <v>29981.32</v>
+      </c>
+      <c r="HC3" s="1" t="n">
+        <v>29903.53</v>
+      </c>
+      <c r="HD3" s="1" t="n">
+        <v>29211.3</v>
+      </c>
+      <c r="HE3" s="1" t="n">
+        <v>28174.75</v>
+      </c>
+      <c r="HF3" s="1" t="n">
+        <v>27713.32</v>
+      </c>
+      <c r="HG3" s="1" t="n">
+        <v>27191.75</v>
+      </c>
+      <c r="HH3" s="1" t="n">
+        <v>26529.35</v>
+      </c>
+      <c r="HI3" s="1" t="n">
+        <v>24256.95</v>
+      </c>
+      <c r="HJ3" s="1" t="n">
+        <v>26349.41</v>
+      </c>
+      <c r="HK3" s="1" t="n">
+        <v>22970.36</v>
+      </c>
+      <c r="HL3" s="1" t="n">
+        <v>22787.51</v>
+      </c>
+      <c r="HM3" s="1" t="n">
+        <v>22708.68</v>
+      </c>
+      <c r="HN3" s="1" t="n">
+        <v>22671.24</v>
+      </c>
+      <c r="HO3" s="1" t="n">
+        <v>20753.51</v>
+      </c>
+      <c r="HP3" s="1" t="n">
+        <v>20763.74</v>
+      </c>
+      <c r="HQ3" s="1" t="n">
+        <v>20227.42</v>
+      </c>
+      <c r="HR3" s="1" t="n">
+        <v>19699.1</v>
+      </c>
+      <c r="HS3" s="1" t="n">
+        <v>47989.24</v>
+      </c>
+      <c r="HT3" s="1" t="n">
+        <v>18519.68</v>
+      </c>
+      <c r="HU3" s="1" t="n">
+        <v>18080.94</v>
+      </c>
+      <c r="HV3" s="1" t="n">
+        <v>31444.98</v>
+      </c>
+      <c r="HW3" s="1" t="n">
+        <v>17156.02</v>
+      </c>
+      <c r="HX3" s="1" t="n">
+        <v>15894.78</v>
+      </c>
+      <c r="HY3" s="1" t="n">
+        <v>15411.03</v>
+      </c>
+      <c r="HZ3" s="1" t="n">
+        <v>15129.67</v>
+      </c>
+      <c r="IA3" s="1" t="n">
+        <v>14788.35</v>
+      </c>
+      <c r="IB3" s="1" t="n">
+        <v>14512.21</v>
+      </c>
+      <c r="IC3" s="1" t="n">
+        <v>14373</v>
+      </c>
+      <c r="ID3" s="1" t="n">
+        <v>12831.05</v>
+      </c>
+      <c r="IE3" s="1" t="n">
+        <v>144672.02</v>
+      </c>
+      <c r="IF3" s="1" t="n">
+        <v>12113.11</v>
+      </c>
+      <c r="IG3" s="1" t="n">
+        <v>11894.77</v>
+      </c>
+      <c r="IH3" s="1" t="n">
+        <v>4340.71</v>
+      </c>
+      <c r="II3" s="1" t="n">
+        <v>17297</v>
+      </c>
+      <c r="IJ3" s="1" t="n">
+        <v>11296.95</v>
+      </c>
+      <c r="IK3" s="1" t="n">
+        <v>11172.42</v>
+      </c>
+      <c r="IL3" s="1" t="n">
+        <v>10949.69</v>
+      </c>
+      <c r="IM3" s="1" t="n">
+        <v>10817.18</v>
+      </c>
+      <c r="IN3" s="1" t="n">
+        <v>10751.53</v>
+      </c>
+      <c r="IO3" s="1" t="n">
+        <v>10255.96</v>
+      </c>
+      <c r="IP3" s="1" t="n">
+        <v>10252.8</v>
+      </c>
+      <c r="IQ3" s="1" t="n">
+        <v>10051.48</v>
+      </c>
+      <c r="IR3" s="1" t="n">
+        <v>9974.91</v>
+      </c>
+      <c r="IS3" s="1" t="n">
+        <v>9747.620000000001</v>
+      </c>
+      <c r="IT3" s="1" t="n">
+        <v>9074.6</v>
+      </c>
+      <c r="IU3" s="1" t="n">
+        <v>8578.940000000001</v>
+      </c>
+      <c r="IV3" s="1" t="n">
+        <v>9706.77</v>
+      </c>
+      <c r="IW3" s="1" t="n">
+        <v>7659.74</v>
+      </c>
+      <c r="IX3" s="1" t="n">
+        <v>25453.52</v>
+      </c>
+      <c r="IY3" s="1" t="n">
+        <v>7130.52</v>
+      </c>
+      <c r="IZ3" s="1" t="n">
+        <v>6887.64</v>
+      </c>
+      <c r="JA3" s="1" t="n">
+        <v>6772.89</v>
+      </c>
+      <c r="JB3" s="1" t="n">
+        <v>6294.66</v>
+      </c>
+      <c r="JC3" s="1" t="n">
+        <v>4472.81</v>
+      </c>
+      <c r="JD3" s="1" t="n">
+        <v>11172.92</v>
+      </c>
+      <c r="JE3" s="1" t="n">
+        <v>5478.54</v>
+      </c>
+      <c r="JF3" s="1" t="n">
+        <v>5281.4</v>
+      </c>
+      <c r="JG3" s="1" t="n">
+        <v>6996.43</v>
+      </c>
+      <c r="JH3" s="1" t="n">
+        <v>5154.27</v>
+      </c>
+      <c r="JI3" s="1" t="n">
+        <v>304353.91</v>
+      </c>
+      <c r="JJ3" s="1" t="n">
+        <v>5084.1</v>
+      </c>
+      <c r="JK3" s="1" t="n">
+        <v>5087.28</v>
+      </c>
+      <c r="JL3" s="1" t="n">
+        <v>5043.86</v>
+      </c>
+      <c r="JM3" s="1" t="n">
+        <v>4970.31</v>
+      </c>
+      <c r="JN3" s="1" t="n">
+        <v>8639.049999999999</v>
+      </c>
+      <c r="JO3" s="1" t="n">
+        <v>4863.59</v>
+      </c>
+      <c r="JP3" s="1" t="n">
+        <v>4774.94</v>
+      </c>
+      <c r="JQ3" s="1" t="n">
+        <v>4771.78</v>
+      </c>
+      <c r="JR3" s="1" t="n">
+        <v>3182.07</v>
+      </c>
+      <c r="JS3" s="1" t="n">
+        <v>4539.76</v>
+      </c>
+      <c r="JT3" s="1" t="n">
+        <v>4353.95</v>
+      </c>
+      <c r="JU3" s="1" t="n">
+        <v>5197.21</v>
+      </c>
+      <c r="JV3" s="1" t="n">
+        <v>3755.76</v>
+      </c>
+      <c r="JW3" s="1" t="n">
+        <v>3714.62</v>
+      </c>
+      <c r="JX3" s="1" t="n">
+        <v>8517.790000000001</v>
+      </c>
+      <c r="JY3" s="1" t="n">
+        <v>3281.13</v>
+      </c>
+      <c r="JZ3" s="1" t="n">
+        <v>3275.23</v>
+      </c>
+      <c r="KA3" s="1" t="n">
+        <v>3201.45</v>
+      </c>
+      <c r="KB3" s="1" t="n">
+        <v>3935.03</v>
+      </c>
+      <c r="KC3" s="1" t="n">
+        <v>3052.85</v>
+      </c>
+      <c r="KD3" s="1" t="n">
+        <v>2990.88</v>
+      </c>
+      <c r="KE3" s="1" t="n">
+        <v>2569.11</v>
+      </c>
+      <c r="KF3" s="1" t="n">
+        <v>2600.84</v>
+      </c>
+      <c r="KG3" s="1" t="n">
+        <v>2566.16</v>
+      </c>
+      <c r="KH3" s="1" t="n">
+        <v>2420.87</v>
+      </c>
+      <c r="KI3" s="1" t="n">
+        <v>2133.16</v>
+      </c>
+      <c r="KJ3" s="1" t="n">
+        <v>1968.05</v>
+      </c>
+      <c r="KK3" s="1" t="n">
+        <v>1936.71</v>
+      </c>
+      <c r="KL3" s="1" t="n">
+        <v>1791.2</v>
+      </c>
+      <c r="KM3" s="1" t="n">
+        <v>1696.51</v>
+      </c>
+      <c r="KN3" s="1" t="n">
+        <v>11650.73</v>
+      </c>
+      <c r="KO3" s="1" t="n">
+        <v>1594.89</v>
+      </c>
+      <c r="KP3" s="1" t="n">
+        <v>1400.01</v>
+      </c>
+      <c r="KQ3" s="1" t="n">
+        <v>1454.51</v>
+      </c>
+      <c r="KR3" s="1" t="n">
+        <v>3051.3</v>
+      </c>
+      <c r="KS3" s="1" t="n">
+        <v>1429.58</v>
+      </c>
+      <c r="KT3" s="1" t="n">
+        <v>1417.84</v>
+      </c>
+      <c r="KU3" s="1" t="n">
+        <v>5831.54</v>
+      </c>
+      <c r="KV3" s="1" t="n">
+        <v>1304.22</v>
+      </c>
+      <c r="KW3" s="1" t="n">
+        <v>26702.16</v>
+      </c>
+      <c r="KX3" s="1" t="n">
+        <v>381.99</v>
+      </c>
+      <c r="KY3" s="1" t="n">
+        <v>1020.83</v>
+      </c>
+      <c r="KZ3" s="1" t="n">
+        <v>1190.1</v>
+      </c>
+      <c r="LA3" s="1" t="n">
+        <v>275.41</v>
+      </c>
+      <c r="LB3" s="1" t="n">
+        <v>1122.94</v>
+      </c>
+      <c r="LC3" s="1" t="n">
+        <v>1119.87</v>
+      </c>
+      <c r="LD3" s="1" t="n">
+        <v>997.5</v>
+      </c>
+      <c r="LE3" s="1" t="n">
+        <v>861.3</v>
+      </c>
+      <c r="LF3" s="1" t="n">
+        <v>893.9400000000001</v>
+      </c>
+      <c r="LG3" s="1" t="n">
+        <v>793.73</v>
+      </c>
+      <c r="LH3" s="1" t="n">
+        <v>850.1799999999999</v>
+      </c>
+      <c r="LI3" s="1" t="n">
+        <v>733.98</v>
+      </c>
+      <c r="LJ3" s="1" t="n">
+        <v>759.1</v>
+      </c>
+      <c r="LK3" s="1" t="n">
+        <v>685.38</v>
+      </c>
+      <c r="LL3" s="1" t="n">
+        <v>614.91</v>
+      </c>
+      <c r="LM3" s="1" t="n">
+        <v>559.92</v>
+      </c>
+      <c r="LN3" s="1" t="n">
+        <v>451.31</v>
+      </c>
+      <c r="LO3" s="1" t="n">
+        <v>449.6</v>
+      </c>
+      <c r="LP3" s="1" t="n">
+        <v>435</v>
+      </c>
+      <c r="LQ3" s="1" t="n">
+        <v>417.78</v>
+      </c>
+      <c r="LR3" s="1" t="n">
+        <v>411.37</v>
+      </c>
+      <c r="LS3" s="1" t="n">
+        <v>408.96</v>
+      </c>
+      <c r="LT3" s="1" t="n">
+        <v>398.52</v>
+      </c>
+      <c r="LU3" s="1" t="n">
+        <v>398.41</v>
+      </c>
+      <c r="LV3" s="1" t="n">
+        <v>301.61</v>
+      </c>
+      <c r="LW3" s="1" t="n">
+        <v>387.88</v>
+      </c>
+      <c r="LX3" s="1" t="n">
+        <v>244.11</v>
+      </c>
+      <c r="LY3" s="1" t="n">
+        <v>199.7</v>
+      </c>
+      <c r="LZ3" s="1" t="n">
+        <v>338.35</v>
+      </c>
+      <c r="MA3" s="1" t="n">
+        <v>433.2</v>
+      </c>
+      <c r="MB3" s="1" t="n">
+        <v>1297.12</v>
+      </c>
+      <c r="MC3" s="1" t="n">
+        <v>305.53</v>
+      </c>
+      <c r="MD3" s="1" t="n">
+        <v>303.08</v>
+      </c>
+      <c r="ME3" s="1" t="n">
+        <v>156.2</v>
+      </c>
+      <c r="MF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="MG3" s="1" t="n">
+        <v>74591.28999999999</v>
+      </c>
+      <c r="MH3" s="1" t="n">
+        <v>248.89</v>
+      </c>
+      <c r="MI3" s="1" t="n">
+        <v>132.85</v>
+      </c>
+      <c r="MJ3" s="1" t="n">
+        <v>216.66</v>
+      </c>
+      <c r="MK3" s="1" t="n">
+        <v>211.35</v>
+      </c>
+      <c r="ML3" s="1" t="n">
+        <v>252.18</v>
+      </c>
+      <c r="MM3" s="1" t="n">
+        <v>199.5</v>
+      </c>
+      <c r="MN3" s="1" t="n">
+        <v>199.49</v>
+      </c>
+      <c r="MO3" s="1" t="n">
+        <v>199.47</v>
+      </c>
+      <c r="MP3" s="1" t="n">
+        <v>199.28</v>
+      </c>
+      <c r="MQ3" s="1" t="n">
+        <v>199.28</v>
+      </c>
+      <c r="MR3" s="1" t="n">
+        <v>195.4</v>
+      </c>
+      <c r="MS3" s="1" t="n">
+        <v>144.29</v>
+      </c>
+      <c r="MT3" s="1" t="n">
+        <v>34.92</v>
+      </c>
+      <c r="MU3" s="1" t="n">
+        <v>20077.65</v>
+      </c>
+      <c r="MV3" s="1" t="n">
+        <v>113.44</v>
+      </c>
+      <c r="MW3" s="1" t="n">
+        <v>111.9</v>
+      </c>
+      <c r="MX3" s="1" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="MY3" s="1" t="n">
+        <v>100.69</v>
+      </c>
+      <c r="MZ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NA3" s="1" t="n">
+        <v>92.54000000000001</v>
+      </c>
+      <c r="NB3" s="1" t="n">
+        <v>57.49</v>
+      </c>
+      <c r="NC3" s="1" t="n">
+        <v>51.15</v>
+      </c>
+      <c r="ND3" s="1" t="n">
+        <v>88.22</v>
+      </c>
+      <c r="NE3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NG3" s="1" t="n">
+        <v>11.97</v>
+      </c>
+      <c r="NH3" s="1" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="NI3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NJ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NK3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NL3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NM3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NN3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NO3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NP3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NQ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NR3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NS3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NT3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NU3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NV3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NW3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NX3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NY3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NZ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OA3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OB3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OC3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OD3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OE3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OG3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OH3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OI3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OJ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OK3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OL3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OM3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="ON3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OO3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OP3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OQ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OR3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OS3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OT3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OU3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OV3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OW3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OX3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OY3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OZ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PA3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PB3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PC3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PD3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PE3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PG3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PH3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PI3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PJ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PK3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PL3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PM3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PN3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PO3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PP3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PQ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PR3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PS3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PT3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PU3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PV3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PW3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PX3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PY3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PZ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="QA3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="QB3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4189,7 +5560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW2"/>
+  <dimension ref="A1:BXW3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4295,6 +5666,44 @@
       </c>
       <c r="M2" s="1" t="n">
         <v>903.806649</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>477159198.56</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>59431221.008</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>12347424.0953</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>8972833.5349</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>3269370.7132</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>1724129.839</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>1051692.3268</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>176784.5229</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>12742.0037</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>8360.57674</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <v>3930.337943</v>
       </c>
     </row>
   </sheetData>
@@ -4308,7 +5717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW2"/>
+  <dimension ref="A1:BXW3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5157,6 +6566,323 @@
         <v>0</v>
       </c>
       <c r="DB2" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>11362893.17644277</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>5798165.383009525</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>3595761.256052385</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>759551.87093175</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>576305.3392889932</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>442902.6259438318</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>325820.2597201968</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>44146.2197843141</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>38492.0139759845</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>20735.115</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <v>15062.4116</v>
+      </c>
+      <c r="N3" s="1" t="n">
+        <v>13031.35616</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>731.097615</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>3943.0207694116</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>1190.3075</v>
+      </c>
+      <c r="R3" s="1" t="n">
+        <v>453.7844069122</v>
+      </c>
+      <c r="S3" s="1" t="n">
+        <v>249.9888</v>
+      </c>
+      <c r="T3" s="1" t="n">
+        <v>99.73321319999999</v>
+      </c>
+      <c r="U3" s="1" t="n">
+        <v>63.363064</v>
+      </c>
+      <c r="V3" s="1" t="n">
+        <v>17.93</v>
+      </c>
+      <c r="W3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB3" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5171,7 +6897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW2"/>
+  <dimension ref="A1:BXW3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5180,10 +6906,316 @@
           <t>Date</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>BTCTHB</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>BTCTHB 7d-Avg</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>XRPTHB</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ETHTHB</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>SOLTHB</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>BCHTHB</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>USDTTHB</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>XLMTHB</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ADATHB</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>POLTHB</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ARBTHB</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>CRVTHB</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>AAVETHB</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>LINKTHB</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>LDOTHB</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>YFITHB</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>CHZTHB</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>BNBTHB</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>SNXTHB</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>SUSHITHB</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>REALXTHB</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>NEARTHB</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>AVAXTHB</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>SANDTHB</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>XAUTTHB</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ZRXTHB</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>SUMXTHB</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>COMPTHB</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ASTERTHB</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>AXSTHB</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>BLUTHB</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>DYDXTHB</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>KNCTHB</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>PENDLETHB</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>TIATHB</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>UNITHB</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>USDCTHB</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>WLDTHB</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>27</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>22777811.28</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>3656214.5</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>1295063.04</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>1113927.77</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>465985.55</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>434891.77</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>330647.95</v>
+      </c>
+      <c r="J3" s="1" t="n">
+        <v>209131.23</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>51937.42</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>42860.59</v>
+      </c>
+      <c r="M3" s="1" t="n">
+        <v>39721.12</v>
+      </c>
+      <c r="N3" s="1" t="n">
+        <v>29533.06</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>27117.95</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>19829.11</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>17356.64</v>
+      </c>
+      <c r="R3" s="1" t="n">
+        <v>15713.17</v>
+      </c>
+      <c r="S3" s="1" t="n">
+        <v>12101.49</v>
+      </c>
+      <c r="T3" s="1" t="n">
+        <v>10009.93</v>
+      </c>
+      <c r="U3" s="1" t="n">
+        <v>8754.68</v>
+      </c>
+      <c r="V3" s="1" t="n">
+        <v>6779.62</v>
+      </c>
+      <c r="W3" s="1" t="n">
+        <v>6038.24</v>
+      </c>
+      <c r="X3" s="1" t="n">
+        <v>4999.99</v>
+      </c>
+      <c r="Y3" s="1" t="n">
+        <v>4658.21</v>
+      </c>
+      <c r="Z3" s="1" t="n">
+        <v>4141.6</v>
+      </c>
+      <c r="AA3" s="1" t="n">
+        <v>1616.55</v>
+      </c>
+      <c r="AB3" s="1" t="n">
+        <v>560.4400000000001</v>
+      </c>
+      <c r="AC3" s="1" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="AD3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update crypto volume snapshot
</commit_message>
<xml_diff>
--- a/crypto_volume.xlsx
+++ b/crypto_volume.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>568660713.29</v>
+        <v>619529776.17</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -481,15 +481,15 @@
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>477159198.56</v>
+        <v>716383579.21</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ETH_THB</t>
+          <t>BTC_THB</t>
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>11362893.17644277</v>
+        <v>4953546.256993227</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="L2" s="1" t="n">
-        <v>22777811.28</v>
+        <v>36245644.96</v>
       </c>
     </row>
     <row r="3">
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>230172684.85</v>
+        <v>248098256.84</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -518,23 +518,23 @@
         </is>
       </c>
       <c r="F3" s="1" t="n">
-        <v>59431221.008</v>
+        <v>75393355.71813001</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BTC_THB</t>
+          <t>ETH_THB</t>
         </is>
       </c>
       <c r="I3" s="1" t="n">
-        <v>5798165.383009525</v>
+        <v>4859159.536246131</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>XRPTHB</t>
+          <t>USDTTHB</t>
         </is>
       </c>
       <c r="L3" s="1" t="n">
-        <v>3656214.5</v>
+        <v>10941725.57</v>
       </c>
     </row>
     <row r="4">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>111501034.51</v>
+        <v>78658560.29000001</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="F4" s="1" t="n">
-        <v>12347424.0953</v>
+        <v>20514427.1186</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -563,15 +563,15 @@
         </is>
       </c>
       <c r="I4" s="1" t="n">
-        <v>3595761.256052385</v>
+        <v>4130046.350622243</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>ETHTHB</t>
+          <t>XRPTHB</t>
         </is>
       </c>
       <c r="L4" s="1" t="n">
-        <v>1295063.04</v>
+        <v>2598733.24</v>
       </c>
     </row>
     <row r="5">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>72974131.79000001</v>
+        <v>33834050.91</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="F5" s="1" t="n">
-        <v>8972833.5349</v>
+        <v>12551433.4178</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -600,15 +600,15 @@
         </is>
       </c>
       <c r="I5" s="1" t="n">
-        <v>759551.87093175</v>
+        <v>450768.0417339354</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>SOLTHB</t>
+          <t>ETHTHB</t>
         </is>
       </c>
       <c r="L5" s="1" t="n">
-        <v>1113927.77</v>
+        <v>849950.76</v>
       </c>
     </row>
     <row r="6">
@@ -617,11 +617,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>THB_SOL</t>
+          <t>THB_DOGE</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>38907350.08</v>
+        <v>25172538.44</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -629,15 +629,15 @@
         </is>
       </c>
       <c r="F6" s="1" t="n">
-        <v>3269370.7132</v>
+        <v>4815890.0662</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>XRP_THB</t>
+          <t>SOL_THB</t>
         </is>
       </c>
       <c r="I6" s="1" t="n">
-        <v>576305.3392889932</v>
+        <v>412110.0657793726</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="L6" s="1" t="n">
-        <v>465985.55</v>
+        <v>701599.66</v>
       </c>
     </row>
     <row r="7"/>
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW3"/>
+  <dimension ref="A1:BXW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5546,6 +5546,1337 @@
         <v>0</v>
       </c>
       <c r="QB3" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>619529776.17</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>248098256.84</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>78658560.29000001</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>33834050.91</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>23912925.23</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>25172538.44</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>6119358.24</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>9784362.279999999</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>8176272.66</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>15356737.17</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>21877821.42</v>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>10538237.89</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>6624532.08</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>1315993.58</v>
+      </c>
+      <c r="Q4" s="1" t="n">
+        <v>7057016.7</v>
+      </c>
+      <c r="R4" s="1" t="n">
+        <v>3070715.41</v>
+      </c>
+      <c r="S4" s="1" t="n">
+        <v>3475737.64</v>
+      </c>
+      <c r="T4" s="1" t="n">
+        <v>3017606.95</v>
+      </c>
+      <c r="U4" s="1" t="n">
+        <v>2741348.49</v>
+      </c>
+      <c r="V4" s="1" t="n">
+        <v>562929.96</v>
+      </c>
+      <c r="W4" s="1" t="n">
+        <v>6074476.7</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>4077416.43</v>
+      </c>
+      <c r="Y4" s="1" t="n">
+        <v>1469917.34</v>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>823293.15</v>
+      </c>
+      <c r="AA4" s="1" t="n">
+        <v>1665241.17</v>
+      </c>
+      <c r="AB4" s="1" t="n">
+        <v>3376338.17</v>
+      </c>
+      <c r="AC4" s="1" t="n">
+        <v>2765472.62</v>
+      </c>
+      <c r="AD4" s="1" t="n">
+        <v>506099.5</v>
+      </c>
+      <c r="AE4" s="1" t="n">
+        <v>853843.76</v>
+      </c>
+      <c r="AF4" s="1" t="n">
+        <v>3212951.12</v>
+      </c>
+      <c r="AG4" s="1" t="n">
+        <v>1532129.16</v>
+      </c>
+      <c r="AH4" s="1" t="n">
+        <v>2536420.06</v>
+      </c>
+      <c r="AI4" s="1" t="n">
+        <v>1869921.6</v>
+      </c>
+      <c r="AJ4" s="1" t="n">
+        <v>2184495.13</v>
+      </c>
+      <c r="AK4" s="1" t="n">
+        <v>977416.65</v>
+      </c>
+      <c r="AL4" s="1" t="n">
+        <v>1625931.94</v>
+      </c>
+      <c r="AM4" s="1" t="n">
+        <v>1587235.59</v>
+      </c>
+      <c r="AN4" s="1" t="n">
+        <v>59892.11</v>
+      </c>
+      <c r="AO4" s="1" t="n">
+        <v>443401.46</v>
+      </c>
+      <c r="AP4" s="1" t="n">
+        <v>1825559.7</v>
+      </c>
+      <c r="AQ4" s="1" t="n">
+        <v>3506265.72</v>
+      </c>
+      <c r="AR4" s="1" t="n">
+        <v>727323.92</v>
+      </c>
+      <c r="AS4" s="1" t="n">
+        <v>255608.8</v>
+      </c>
+      <c r="AT4" s="1" t="n">
+        <v>1433132.06</v>
+      </c>
+      <c r="AU4" s="1" t="n">
+        <v>1638828.95</v>
+      </c>
+      <c r="AV4" s="1" t="n">
+        <v>3986319.85</v>
+      </c>
+      <c r="AW4" s="1" t="n">
+        <v>1177849.94</v>
+      </c>
+      <c r="AX4" s="1" t="n">
+        <v>1392402.44</v>
+      </c>
+      <c r="AY4" s="1" t="n">
+        <v>178007.5</v>
+      </c>
+      <c r="AZ4" s="1" t="n">
+        <v>450098.43</v>
+      </c>
+      <c r="BA4" s="1" t="n">
+        <v>326843.97</v>
+      </c>
+      <c r="BB4" s="1" t="n">
+        <v>1283865.4</v>
+      </c>
+      <c r="BC4" s="1" t="n">
+        <v>853761.55</v>
+      </c>
+      <c r="BD4" s="1" t="n">
+        <v>693061.41</v>
+      </c>
+      <c r="BE4" s="1" t="n">
+        <v>608846.75</v>
+      </c>
+      <c r="BF4" s="1" t="n">
+        <v>1043126.62</v>
+      </c>
+      <c r="BG4" s="1" t="n">
+        <v>127556.6</v>
+      </c>
+      <c r="BH4" s="1" t="n">
+        <v>862014.58</v>
+      </c>
+      <c r="BI4" s="1" t="n">
+        <v>273599.83</v>
+      </c>
+      <c r="BJ4" s="1" t="n">
+        <v>598807.97</v>
+      </c>
+      <c r="BK4" s="1" t="n">
+        <v>515499.66</v>
+      </c>
+      <c r="BL4" s="1" t="n">
+        <v>997383.77</v>
+      </c>
+      <c r="BM4" s="1" t="n">
+        <v>165124.52</v>
+      </c>
+      <c r="BN4" s="1" t="n">
+        <v>342677.7</v>
+      </c>
+      <c r="BO4" s="1" t="n">
+        <v>122327.07</v>
+      </c>
+      <c r="BP4" s="1" t="n">
+        <v>137811.89</v>
+      </c>
+      <c r="BQ4" s="1" t="n">
+        <v>313476.61</v>
+      </c>
+      <c r="BR4" s="1" t="n">
+        <v>606043.35</v>
+      </c>
+      <c r="BS4" s="1" t="n">
+        <v>1628867.41</v>
+      </c>
+      <c r="BT4" s="1" t="n">
+        <v>73056.78999999999</v>
+      </c>
+      <c r="BU4" s="1" t="n">
+        <v>1682401.51</v>
+      </c>
+      <c r="BV4" s="1" t="n">
+        <v>1614766.74</v>
+      </c>
+      <c r="BW4" s="1" t="n">
+        <v>11927.56</v>
+      </c>
+      <c r="BX4" s="1" t="n">
+        <v>38531.51</v>
+      </c>
+      <c r="BY4" s="1" t="n">
+        <v>337578.06</v>
+      </c>
+      <c r="BZ4" s="1" t="n">
+        <v>54049.06</v>
+      </c>
+      <c r="CA4" s="1" t="n">
+        <v>231099.71</v>
+      </c>
+      <c r="CB4" s="1" t="n">
+        <v>1165408.26</v>
+      </c>
+      <c r="CC4" s="1" t="n">
+        <v>1658482.54</v>
+      </c>
+      <c r="CD4" s="1" t="n">
+        <v>720145.29</v>
+      </c>
+      <c r="CE4" s="1" t="n">
+        <v>93701.37</v>
+      </c>
+      <c r="CF4" s="1" t="n">
+        <v>100835.82</v>
+      </c>
+      <c r="CG4" s="1" t="n">
+        <v>849823.28</v>
+      </c>
+      <c r="CH4" s="1" t="n">
+        <v>6372.18</v>
+      </c>
+      <c r="CI4" s="1" t="n">
+        <v>78816.67999999999</v>
+      </c>
+      <c r="CJ4" s="1" t="n">
+        <v>1646939.48</v>
+      </c>
+      <c r="CK4" s="1" t="n">
+        <v>445561.41</v>
+      </c>
+      <c r="CL4" s="1" t="n">
+        <v>194303.95</v>
+      </c>
+      <c r="CM4" s="1" t="n">
+        <v>31587.24</v>
+      </c>
+      <c r="CN4" s="1" t="n">
+        <v>311438.01</v>
+      </c>
+      <c r="CO4" s="1" t="n">
+        <v>1008213.67</v>
+      </c>
+      <c r="CP4" s="1" t="n">
+        <v>147757.7</v>
+      </c>
+      <c r="CQ4" s="1" t="n">
+        <v>864202.85</v>
+      </c>
+      <c r="CR4" s="1" t="n">
+        <v>207180.09</v>
+      </c>
+      <c r="CS4" s="1" t="n">
+        <v>43296.32</v>
+      </c>
+      <c r="CT4" s="1" t="n">
+        <v>19529.7</v>
+      </c>
+      <c r="CU4" s="1" t="n">
+        <v>246667.8</v>
+      </c>
+      <c r="CV4" s="1" t="n">
+        <v>264491.18</v>
+      </c>
+      <c r="CW4" s="1" t="n">
+        <v>600281.98</v>
+      </c>
+      <c r="CX4" s="1" t="n">
+        <v>225881.9</v>
+      </c>
+      <c r="CY4" s="1" t="n">
+        <v>3864</v>
+      </c>
+      <c r="CZ4" s="1" t="n">
+        <v>271226.07</v>
+      </c>
+      <c r="DA4" s="1" t="n">
+        <v>7587.43</v>
+      </c>
+      <c r="DB4" s="1" t="n">
+        <v>148836.52</v>
+      </c>
+      <c r="DC4" s="1" t="n">
+        <v>23870.69</v>
+      </c>
+      <c r="DD4" s="1" t="n">
+        <v>276884.7</v>
+      </c>
+      <c r="DE4" s="1" t="n">
+        <v>154739.74</v>
+      </c>
+      <c r="DF4" s="1" t="n">
+        <v>196756.47</v>
+      </c>
+      <c r="DG4" s="1" t="n">
+        <v>658728.48</v>
+      </c>
+      <c r="DH4" s="1" t="n">
+        <v>489340.66</v>
+      </c>
+      <c r="DI4" s="1" t="n">
+        <v>86131.63</v>
+      </c>
+      <c r="DJ4" s="1" t="n">
+        <v>43125.59</v>
+      </c>
+      <c r="DK4" s="1" t="n">
+        <v>360299.35</v>
+      </c>
+      <c r="DL4" s="1" t="n">
+        <v>85385.24000000001</v>
+      </c>
+      <c r="DM4" s="1" t="n">
+        <v>260027.89</v>
+      </c>
+      <c r="DN4" s="1" t="n">
+        <v>108155.38</v>
+      </c>
+      <c r="DO4" s="1" t="n">
+        <v>362523.76</v>
+      </c>
+      <c r="DP4" s="1" t="n">
+        <v>20031.91</v>
+      </c>
+      <c r="DQ4" s="1" t="n">
+        <v>28533.06</v>
+      </c>
+      <c r="DR4" s="1" t="n">
+        <v>229101.22</v>
+      </c>
+      <c r="DS4" s="1" t="n">
+        <v>29353.73</v>
+      </c>
+      <c r="DT4" s="1" t="n">
+        <v>192697.44</v>
+      </c>
+      <c r="DU4" s="1" t="n">
+        <v>135243.2</v>
+      </c>
+      <c r="DV4" s="1" t="n">
+        <v>216063.76</v>
+      </c>
+      <c r="DW4" s="1" t="n">
+        <v>2124.15</v>
+      </c>
+      <c r="DX4" s="1" t="n">
+        <v>413377.05</v>
+      </c>
+      <c r="DY4" s="1" t="n">
+        <v>6339.34</v>
+      </c>
+      <c r="DZ4" s="1" t="n">
+        <v>86196.39999999999</v>
+      </c>
+      <c r="EA4" s="1" t="n">
+        <v>15693.39</v>
+      </c>
+      <c r="EB4" s="1" t="n">
+        <v>2312.59</v>
+      </c>
+      <c r="EC4" s="1" t="n">
+        <v>22743.61</v>
+      </c>
+      <c r="ED4" s="1" t="n">
+        <v>402277.02</v>
+      </c>
+      <c r="EE4" s="1" t="n">
+        <v>96475.47</v>
+      </c>
+      <c r="EF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="EG4" s="1" t="n">
+        <v>26849.53</v>
+      </c>
+      <c r="EH4" s="1" t="n">
+        <v>598.6799999999999</v>
+      </c>
+      <c r="EI4" s="1" t="n">
+        <v>105390.61</v>
+      </c>
+      <c r="EJ4" s="1" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="EK4" s="1" t="n">
+        <v>205170.53</v>
+      </c>
+      <c r="EL4" s="1" t="n">
+        <v>99465.34</v>
+      </c>
+      <c r="EM4" s="1" t="n">
+        <v>102428.18</v>
+      </c>
+      <c r="EN4" s="1" t="n">
+        <v>19256.18</v>
+      </c>
+      <c r="EO4" s="1" t="n">
+        <v>138874.69</v>
+      </c>
+      <c r="EP4" s="1" t="n">
+        <v>45908.27</v>
+      </c>
+      <c r="EQ4" s="1" t="n">
+        <v>662.3200000000001</v>
+      </c>
+      <c r="ER4" s="1" t="n">
+        <v>22007.76</v>
+      </c>
+      <c r="ES4" s="1" t="n">
+        <v>5468.67</v>
+      </c>
+      <c r="ET4" s="1" t="n">
+        <v>89880.89999999999</v>
+      </c>
+      <c r="EU4" s="1" t="n">
+        <v>45636.98</v>
+      </c>
+      <c r="EV4" s="1" t="n">
+        <v>26814.17</v>
+      </c>
+      <c r="EW4" s="1" t="n">
+        <v>101453.48</v>
+      </c>
+      <c r="EX4" s="1" t="n">
+        <v>309009.11</v>
+      </c>
+      <c r="EY4" s="1" t="n">
+        <v>25705.42</v>
+      </c>
+      <c r="EZ4" s="1" t="n">
+        <v>99.75</v>
+      </c>
+      <c r="FA4" s="1" t="n">
+        <v>66407.73</v>
+      </c>
+      <c r="FB4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC4" s="1" t="n">
+        <v>229508.18</v>
+      </c>
+      <c r="FD4" s="1" t="n">
+        <v>1657560.14</v>
+      </c>
+      <c r="FE4" s="1" t="n">
+        <v>941605.99</v>
+      </c>
+      <c r="FF4" s="1" t="n">
+        <v>48879.86</v>
+      </c>
+      <c r="FG4" s="1" t="n">
+        <v>165409.36</v>
+      </c>
+      <c r="FH4" s="1" t="n">
+        <v>29289.71</v>
+      </c>
+      <c r="FI4" s="1" t="n">
+        <v>61319.82</v>
+      </c>
+      <c r="FJ4" s="1" t="n">
+        <v>61598.86</v>
+      </c>
+      <c r="FK4" s="1" t="n">
+        <v>70642.11</v>
+      </c>
+      <c r="FL4" s="1" t="n">
+        <v>77898.60000000001</v>
+      </c>
+      <c r="FM4" s="1" t="n">
+        <v>64856.01</v>
+      </c>
+      <c r="FN4" s="1" t="n">
+        <v>123727.27</v>
+      </c>
+      <c r="FO4" s="1" t="n">
+        <v>1234.4</v>
+      </c>
+      <c r="FP4" s="1" t="n">
+        <v>2209.86</v>
+      </c>
+      <c r="FQ4" s="1" t="n">
+        <v>532587.58</v>
+      </c>
+      <c r="FR4" s="1" t="n">
+        <v>18939.1</v>
+      </c>
+      <c r="FS4" s="1" t="n">
+        <v>834210.05</v>
+      </c>
+      <c r="FT4" s="1" t="n">
+        <v>135.25</v>
+      </c>
+      <c r="FU4" s="1" t="n">
+        <v>35867.93</v>
+      </c>
+      <c r="FV4" s="1" t="n">
+        <v>88352.22</v>
+      </c>
+      <c r="FW4" s="1" t="n">
+        <v>16073.5</v>
+      </c>
+      <c r="FX4" s="1" t="n">
+        <v>122643.4</v>
+      </c>
+      <c r="FY4" s="1" t="n">
+        <v>143122.91</v>
+      </c>
+      <c r="FZ4" s="1" t="n">
+        <v>1735.18</v>
+      </c>
+      <c r="GA4" s="1" t="n">
+        <v>73872.25</v>
+      </c>
+      <c r="GB4" s="1" t="n">
+        <v>637.63</v>
+      </c>
+      <c r="GC4" s="1" t="n">
+        <v>5101.84</v>
+      </c>
+      <c r="GD4" s="1" t="n">
+        <v>1878.05</v>
+      </c>
+      <c r="GE4" s="1" t="n">
+        <v>105103.64</v>
+      </c>
+      <c r="GF4" s="1" t="n">
+        <v>27044.54</v>
+      </c>
+      <c r="GG4" s="1" t="n">
+        <v>104488.28</v>
+      </c>
+      <c r="GH4" s="1" t="n">
+        <v>178341.25</v>
+      </c>
+      <c r="GI4" s="1" t="n">
+        <v>36368.86</v>
+      </c>
+      <c r="GJ4" s="1" t="n">
+        <v>4150.94</v>
+      </c>
+      <c r="GK4" s="1" t="n">
+        <v>519862.31</v>
+      </c>
+      <c r="GL4" s="1" t="n">
+        <v>22852.63</v>
+      </c>
+      <c r="GM4" s="1" t="n">
+        <v>78997.87</v>
+      </c>
+      <c r="GN4" s="1" t="n">
+        <v>22530.45</v>
+      </c>
+      <c r="GO4" s="1" t="n">
+        <v>379816.5</v>
+      </c>
+      <c r="GP4" s="1" t="n">
+        <v>53424.86</v>
+      </c>
+      <c r="GQ4" s="1" t="n">
+        <v>41599.55</v>
+      </c>
+      <c r="GR4" s="1" t="n">
+        <v>2817.02</v>
+      </c>
+      <c r="GS4" s="1" t="n">
+        <v>34143.13</v>
+      </c>
+      <c r="GT4" s="1" t="n">
+        <v>342522.57</v>
+      </c>
+      <c r="GU4" s="1" t="n">
+        <v>27534.95</v>
+      </c>
+      <c r="GV4" s="1" t="n">
+        <v>328255.32</v>
+      </c>
+      <c r="GW4" s="1" t="n">
+        <v>36869.97</v>
+      </c>
+      <c r="GX4" s="1" t="n">
+        <v>45556.46</v>
+      </c>
+      <c r="GY4" s="1" t="n">
+        <v>278100.44</v>
+      </c>
+      <c r="GZ4" s="1" t="n">
+        <v>942.25</v>
+      </c>
+      <c r="HA4" s="1" t="n">
+        <v>73835.96000000001</v>
+      </c>
+      <c r="HB4" s="1" t="n">
+        <v>99.73999999999999</v>
+      </c>
+      <c r="HC4" s="1" t="n">
+        <v>44517.49</v>
+      </c>
+      <c r="HD4" s="1" t="n">
+        <v>19901.72</v>
+      </c>
+      <c r="HE4" s="1" t="n">
+        <v>15116.59</v>
+      </c>
+      <c r="HF4" s="1" t="n">
+        <v>4387.77</v>
+      </c>
+      <c r="HG4" s="1" t="n">
+        <v>16950.36</v>
+      </c>
+      <c r="HH4" s="1" t="n">
+        <v>38.19</v>
+      </c>
+      <c r="HI4" s="1" t="n">
+        <v>36378.06</v>
+      </c>
+      <c r="HJ4" s="1" t="n">
+        <v>22134.33</v>
+      </c>
+      <c r="HK4" s="1" t="n">
+        <v>76728.41</v>
+      </c>
+      <c r="HL4" s="1" t="n">
+        <v>167725.97</v>
+      </c>
+      <c r="HM4" s="1" t="n">
+        <v>2695.75</v>
+      </c>
+      <c r="HN4" s="1" t="n">
+        <v>241214.65</v>
+      </c>
+      <c r="HO4" s="1" t="n">
+        <v>25608.29</v>
+      </c>
+      <c r="HP4" s="1" t="n">
+        <v>147152.48</v>
+      </c>
+      <c r="HQ4" s="1" t="n">
+        <v>16061.68</v>
+      </c>
+      <c r="HR4" s="1" t="n">
+        <v>12648.94</v>
+      </c>
+      <c r="HS4" s="1" t="n">
+        <v>176644.87</v>
+      </c>
+      <c r="HT4" s="1" t="n">
+        <v>52397.2</v>
+      </c>
+      <c r="HU4" s="1" t="n">
+        <v>693.8099999999999</v>
+      </c>
+      <c r="HV4" s="1" t="n">
+        <v>250594.66</v>
+      </c>
+      <c r="HW4" s="1" t="n">
+        <v>1360.57</v>
+      </c>
+      <c r="HX4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="HY4" s="1" t="n">
+        <v>38794.93</v>
+      </c>
+      <c r="HZ4" s="1" t="n">
+        <v>23.49</v>
+      </c>
+      <c r="IA4" s="1" t="n">
+        <v>1951.28</v>
+      </c>
+      <c r="IB4" s="1" t="n">
+        <v>3009.52</v>
+      </c>
+      <c r="IC4" s="1" t="n">
+        <v>4931.65</v>
+      </c>
+      <c r="ID4" s="1" t="n">
+        <v>29795.35</v>
+      </c>
+      <c r="IE4" s="1" t="n">
+        <v>55348.16</v>
+      </c>
+      <c r="IF4" s="1" t="n">
+        <v>8080.83</v>
+      </c>
+      <c r="IG4" s="1" t="n">
+        <v>112246.81</v>
+      </c>
+      <c r="IH4" s="1" t="n">
+        <v>1437.42</v>
+      </c>
+      <c r="II4" s="1" t="n">
+        <v>93490.67999999999</v>
+      </c>
+      <c r="IJ4" s="1" t="n">
+        <v>22275.84</v>
+      </c>
+      <c r="IK4" s="1" t="n">
+        <v>25980.84</v>
+      </c>
+      <c r="IL4" s="1" t="n">
+        <v>4473</v>
+      </c>
+      <c r="IM4" s="1" t="n">
+        <v>30924</v>
+      </c>
+      <c r="IN4" s="1" t="n">
+        <v>2204.47</v>
+      </c>
+      <c r="IO4" s="1" t="n">
+        <v>144851.12</v>
+      </c>
+      <c r="IP4" s="1" t="n">
+        <v>1348.69</v>
+      </c>
+      <c r="IQ4" s="1" t="n">
+        <v>3859</v>
+      </c>
+      <c r="IR4" s="1" t="n">
+        <v>9974.91</v>
+      </c>
+      <c r="IS4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="IT4" s="1" t="n">
+        <v>8796.02</v>
+      </c>
+      <c r="IU4" s="1" t="n">
+        <v>12793.17</v>
+      </c>
+      <c r="IV4" s="1" t="n">
+        <v>17198.86</v>
+      </c>
+      <c r="IW4" s="1" t="n">
+        <v>304174.5</v>
+      </c>
+      <c r="IX4" s="1" t="n">
+        <v>28865.33</v>
+      </c>
+      <c r="IY4" s="1" t="n">
+        <v>7133.07</v>
+      </c>
+      <c r="IZ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA4" s="1" t="n">
+        <v>1513.61</v>
+      </c>
+      <c r="JB4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JC4" s="1" t="n">
+        <v>12218.31</v>
+      </c>
+      <c r="JD4" s="1" t="n">
+        <v>8204.290000000001</v>
+      </c>
+      <c r="JE4" s="1" t="n">
+        <v>39220.44</v>
+      </c>
+      <c r="JF4" s="1" t="n">
+        <v>8187.33</v>
+      </c>
+      <c r="JG4" s="1" t="n">
+        <v>15648</v>
+      </c>
+      <c r="JH4" s="1" t="n">
+        <v>5154.27</v>
+      </c>
+      <c r="JI4" s="1" t="n">
+        <v>71142.39</v>
+      </c>
+      <c r="JJ4" s="1" t="n">
+        <v>23.16</v>
+      </c>
+      <c r="JK4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JL4" s="1" t="n">
+        <v>5043.86</v>
+      </c>
+      <c r="JM4" s="1" t="n">
+        <v>3160.03</v>
+      </c>
+      <c r="JN4" s="1" t="n">
+        <v>10221.77</v>
+      </c>
+      <c r="JO4" s="1" t="n">
+        <v>4863.59</v>
+      </c>
+      <c r="JP4" s="1" t="n">
+        <v>1028.47</v>
+      </c>
+      <c r="JQ4" s="1" t="n">
+        <v>199.31</v>
+      </c>
+      <c r="JR4" s="1" t="n">
+        <v>3706.13</v>
+      </c>
+      <c r="JS4" s="1" t="n">
+        <v>60285.37</v>
+      </c>
+      <c r="JT4" s="1" t="n">
+        <v>199.5</v>
+      </c>
+      <c r="JU4" s="1" t="n">
+        <v>15581.6</v>
+      </c>
+      <c r="JV4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JW4" s="1" t="n">
+        <v>3714.62</v>
+      </c>
+      <c r="JX4" s="1" t="n">
+        <v>99.75</v>
+      </c>
+      <c r="JY4" s="1" t="n">
+        <v>22299.37</v>
+      </c>
+      <c r="JZ4" s="1" t="n">
+        <v>6135.33</v>
+      </c>
+      <c r="KA4" s="1" t="n">
+        <v>193118.87</v>
+      </c>
+      <c r="KB4" s="1" t="n">
+        <v>13434.1</v>
+      </c>
+      <c r="KC4" s="1" t="n">
+        <v>9159.379999999999</v>
+      </c>
+      <c r="KD4" s="1" t="n">
+        <v>398.34</v>
+      </c>
+      <c r="KE4" s="1" t="n">
+        <v>355.9</v>
+      </c>
+      <c r="KF4" s="1" t="n">
+        <v>401.82</v>
+      </c>
+      <c r="KG4" s="1" t="n">
+        <v>33547.68</v>
+      </c>
+      <c r="KH4" s="1" t="n">
+        <v>57840.96</v>
+      </c>
+      <c r="KI4" s="1" t="n">
+        <v>40320.31</v>
+      </c>
+      <c r="KJ4" s="1" t="n">
+        <v>199.5</v>
+      </c>
+      <c r="KK4" s="1" t="n">
+        <v>198.61</v>
+      </c>
+      <c r="KL4" s="1" t="n">
+        <v>1791.2</v>
+      </c>
+      <c r="KM4" s="1" t="n">
+        <v>29745.39</v>
+      </c>
+      <c r="KN4" s="1" t="n">
+        <v>43109.78</v>
+      </c>
+      <c r="KO4" s="1" t="n">
+        <v>56518.99</v>
+      </c>
+      <c r="KP4" s="1" t="n">
+        <v>1022.04</v>
+      </c>
+      <c r="KQ4" s="1" t="n">
+        <v>8289.67</v>
+      </c>
+      <c r="KR4" s="1" t="n">
+        <v>76.20999999999999</v>
+      </c>
+      <c r="KS4" s="1" t="n">
+        <v>688009.0600000001</v>
+      </c>
+      <c r="KT4" s="1" t="n">
+        <v>100873.61</v>
+      </c>
+      <c r="KU4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="KV4" s="1" t="n">
+        <v>99.75</v>
+      </c>
+      <c r="KW4" s="1" t="n">
+        <v>466.21</v>
+      </c>
+      <c r="KX4" s="1" t="n">
+        <v>14.96</v>
+      </c>
+      <c r="KY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="KZ4" s="1" t="n">
+        <v>20362.5</v>
+      </c>
+      <c r="LA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="LB4" s="1" t="n">
+        <v>815179.04</v>
+      </c>
+      <c r="LC4" s="1" t="n">
+        <v>584.72</v>
+      </c>
+      <c r="LD4" s="1" t="n">
+        <v>135562.43</v>
+      </c>
+      <c r="LE4" s="1" t="n">
+        <v>19145.99</v>
+      </c>
+      <c r="LF4" s="1" t="n">
+        <v>199.46</v>
+      </c>
+      <c r="LG4" s="1" t="n">
+        <v>2166.8</v>
+      </c>
+      <c r="LH4" s="1" t="n">
+        <v>850.1799999999999</v>
+      </c>
+      <c r="LI4" s="1" t="n">
+        <v>13114.72</v>
+      </c>
+      <c r="LJ4" s="1" t="n">
+        <v>1771.64</v>
+      </c>
+      <c r="LK4" s="1" t="n">
+        <v>629.6900000000001</v>
+      </c>
+      <c r="LL4" s="1" t="n">
+        <v>152675.46</v>
+      </c>
+      <c r="LM4" s="1" t="n">
+        <v>559.92</v>
+      </c>
+      <c r="LN4" s="1" t="n">
+        <v>451.31</v>
+      </c>
+      <c r="LO4" s="1" t="n">
+        <v>449.6</v>
+      </c>
+      <c r="LP4" s="1" t="n">
+        <v>10337.43</v>
+      </c>
+      <c r="LQ4" s="1" t="n">
+        <v>110.83</v>
+      </c>
+      <c r="LR4" s="1" t="n">
+        <v>3217.77</v>
+      </c>
+      <c r="LS4" s="1" t="n">
+        <v>185.79</v>
+      </c>
+      <c r="LT4" s="1" t="n">
+        <v>997.38</v>
+      </c>
+      <c r="LU4" s="1" t="n">
+        <v>398.41</v>
+      </c>
+      <c r="LV4" s="1" t="n">
+        <v>1569.29</v>
+      </c>
+      <c r="LW4" s="1" t="n">
+        <v>44830.93</v>
+      </c>
+      <c r="LX4" s="1" t="n">
+        <v>929.67</v>
+      </c>
+      <c r="LY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="LZ4" s="1" t="n">
+        <v>10086.22</v>
+      </c>
+      <c r="MA4" s="1" t="n">
+        <v>253.88</v>
+      </c>
+      <c r="MB4" s="1" t="n">
+        <v>2780.11</v>
+      </c>
+      <c r="MC4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="MD4" s="1" t="n">
+        <v>31450.04</v>
+      </c>
+      <c r="ME4" s="1" t="n">
+        <v>487.83</v>
+      </c>
+      <c r="MF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="MG4" s="1" t="n">
+        <v>223184.58</v>
+      </c>
+      <c r="MH4" s="1" t="n">
+        <v>5064.07</v>
+      </c>
+      <c r="MI4" s="1" t="n">
+        <v>8544.66</v>
+      </c>
+      <c r="MJ4" s="1" t="n">
+        <v>7423.97</v>
+      </c>
+      <c r="MK4" s="1" t="n">
+        <v>1187.34</v>
+      </c>
+      <c r="ML4" s="1" t="n">
+        <v>362.16</v>
+      </c>
+      <c r="MM4" s="1" t="n">
+        <v>200.33</v>
+      </c>
+      <c r="MN4" s="1" t="n">
+        <v>199.49</v>
+      </c>
+      <c r="MO4" s="1" t="n">
+        <v>199.47</v>
+      </c>
+      <c r="MP4" s="1" t="n">
+        <v>17049.92</v>
+      </c>
+      <c r="MQ4" s="1" t="n">
+        <v>199.28</v>
+      </c>
+      <c r="MR4" s="1" t="n">
+        <v>18229.31</v>
+      </c>
+      <c r="MS4" s="1" t="n">
+        <v>269.7</v>
+      </c>
+      <c r="MT4" s="1" t="n">
+        <v>10695.41</v>
+      </c>
+      <c r="MU4" s="1" t="n">
+        <v>84085.89999999999</v>
+      </c>
+      <c r="MV4" s="1" t="n">
+        <v>4987.52</v>
+      </c>
+      <c r="MW4" s="1" t="n">
+        <v>5087.26</v>
+      </c>
+      <c r="MX4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="MY4" s="1" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="MZ4" s="1" t="n">
+        <v>12764.38</v>
+      </c>
+      <c r="NA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NB4" s="1" t="n">
+        <v>99.75</v>
+      </c>
+      <c r="NC4" s="1" t="n">
+        <v>9142.620000000001</v>
+      </c>
+      <c r="ND4" s="1" t="n">
+        <v>169392.28</v>
+      </c>
+      <c r="NE4" s="1" t="n">
+        <v>1646.62</v>
+      </c>
+      <c r="NF4" s="1" t="n">
+        <v>549.75</v>
+      </c>
+      <c r="NG4" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="NH4" s="1" t="n">
+        <v>21909.38</v>
+      </c>
+      <c r="NI4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NJ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NK4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NL4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NM4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NN4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NO4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NP4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NQ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NR4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NS4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NT4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NU4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NV4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NW4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NX4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NZ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OB4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OC4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OD4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OE4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OG4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OH4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OI4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OJ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OK4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OL4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OM4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="ON4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OO4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OP4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OQ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OR4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OS4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OT4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OU4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OV4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OW4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OX4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="OZ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PB4" s="1" t="n">
+        <v>498.74</v>
+      </c>
+      <c r="PC4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PD4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PE4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PG4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PH4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PI4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PJ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PK4" s="1" t="n">
+        <v>9859.5</v>
+      </c>
+      <c r="PL4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PM4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PN4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PO4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PP4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PQ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PR4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PS4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PT4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PU4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PV4" s="1" t="n">
+        <v>713.37</v>
+      </c>
+      <c r="PW4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PX4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PZ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="QA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="QB4" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5560,7 +6891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW3"/>
+  <dimension ref="A1:BXW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5704,6 +7035,44 @@
       </c>
       <c r="M3" s="1" t="n">
         <v>3930.337943</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>716383579.21</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>75393355.71813001</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>20514427.1186</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>12551433.4178</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>4815890.0662</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>3202469.9998</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>3717558.3548</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>17727.1743</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>34306.2575</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>2406.2268</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>21670.594923</v>
       </c>
     </row>
   </sheetData>
@@ -5717,7 +7086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW3"/>
+  <dimension ref="A1:BXW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6883,6 +8252,323 @@
         <v>0</v>
       </c>
       <c r="DB3" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>4859159.536246131</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>4953546.256993227</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>4130046.350622243</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>450768.0417339354</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>153110.837</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>412110.0657793726</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>102482.6571023</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>28119.22</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>65188.8275766628</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>56.08</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>6.1055</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>202.09</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>99.00360000000001</v>
+      </c>
+      <c r="Q4" s="1" t="n">
+        <v>8385.18833635</v>
+      </c>
+      <c r="R4" s="1" t="n">
+        <v>3982.065004</v>
+      </c>
+      <c r="S4" s="1" t="n">
+        <v>181.4858</v>
+      </c>
+      <c r="T4" s="1" t="n">
+        <v>49.725</v>
+      </c>
+      <c r="U4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="1" t="n">
+        <v>167.02335</v>
+      </c>
+      <c r="AE4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI4" s="1" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="BJ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX4" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="CY4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB4" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6897,7 +8583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW3"/>
+  <dimension ref="A1:BXW4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7216,6 +8902,122 @@
       </c>
       <c r="AM3" s="1" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>36245644.96</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>2598733.24</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>849950.76</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>335367.25</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>701599.66</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>10941725.57</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>251047.86</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>302812.17</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>1296.22</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1" t="n">
+        <v>68988.31</v>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>19601.58</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>507</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>3568.93</v>
+      </c>
+      <c r="Q4" s="1" t="n">
+        <v>3734.4</v>
+      </c>
+      <c r="R4" s="1" t="n">
+        <v>18624.65</v>
+      </c>
+      <c r="S4" s="1" t="n">
+        <v>48523.7</v>
+      </c>
+      <c r="T4" s="1" t="n">
+        <v>14679.77</v>
+      </c>
+      <c r="U4" s="1" t="n">
+        <v>3130</v>
+      </c>
+      <c r="V4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="1" t="n">
+        <v>509581.38</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>253467.65</v>
+      </c>
+      <c r="AA4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="1" t="n">
+        <v>501.5</v>
+      </c>
+      <c r="AC4" s="1" t="n">
+        <v>3930.68</v>
+      </c>
+      <c r="AD4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="1" t="n">
+        <v>42819.57</v>
+      </c>
+      <c r="AI4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="1" t="n">
+        <v>101601.13</v>
+      </c>
+      <c r="AL4" s="1" t="n">
+        <v>33559.37</v>
+      </c>
+      <c r="AM4" s="1" t="n">
+        <v>5000.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>